<commit_message>
The first four level, fix a few bugs
</commit_message>
<xml_diff>
--- a/Src/Assets/Common/Tables/Tables/Levels.xlsx
+++ b/Src/Assets/Common/Tables/Tables/Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\Common\Tables\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6867075D-A563-474B-A0D9-C92C654A91BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4038F88-340B-493E-8C04-90F59B3F7BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Character" sheetId="2" r:id="rId1"/>
@@ -1362,10 +1362,6 @@
   </si>
   <si>
     <t>[]</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>["Save Me!!!"]</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
@@ -1980,6 +1976,32 @@
   <si>
     <t>PreviousLevel</t>
     <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>["Save</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> Me"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2297,7 +2319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2467,9 +2489,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3207,13 +3226,13 @@
         <v>2</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F1" s="22" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H1" s="22" t="s">
         <v>8</v>
@@ -3278,7 +3297,7 @@
         <v>250</v>
       </c>
       <c r="M2" s="26" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N2" s="26" t="s">
         <v>359</v>
@@ -3324,7 +3343,7 @@
         <v>12</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N3" s="11" t="s">
         <v>359</v>
@@ -3368,7 +3387,7 @@
         <v>12</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>359</v>
@@ -3414,7 +3433,7 @@
         <v>12</v>
       </c>
       <c r="M5" s="16" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N5" s="11" t="s">
         <v>359</v>
@@ -3437,7 +3456,7 @@
       <c r="E6" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="F6" s="61" t="b">
+      <c r="F6" s="60" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="6"/>
@@ -3458,10 +3477,10 @@
         <v>12</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>421</v>
-      </c>
-      <c r="N6" s="58" t="s">
-        <v>360</v>
+        <v>420</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>489</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
@@ -3488,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="29" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
@@ -3504,10 +3523,10 @@
         <v>12</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N7" s="29" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3548,10 +3567,10 @@
         <v>250</v>
       </c>
       <c r="M8" s="33" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N8" s="33" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="O8" s="33"/>
       <c r="P8" s="33"/>
@@ -3595,7 +3614,7 @@
         <v>12</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N9" s="11" t="s">
         <v>359</v>
@@ -3639,7 +3658,7 @@
         <v>12</v>
       </c>
       <c r="M10" s="32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N10" s="32" t="s">
         <v>359</v>
@@ -3686,7 +3705,7 @@
         <v>12</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N11" s="11" t="s">
         <v>359</v>
@@ -3730,7 +3749,7 @@
         <v>12</v>
       </c>
       <c r="M12" s="32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N12" s="32" t="s">
         <v>359</v>
@@ -3779,10 +3798,10 @@
         <v>12</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N13" s="29" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3823,10 +3842,10 @@
         <v>250</v>
       </c>
       <c r="M14" s="33" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N14" s="33" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="O14" s="33"/>
       <c r="P14" s="33"/>
@@ -3872,10 +3891,10 @@
         <v>246</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N15" s="29" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3918,10 +3937,10 @@
         <v>12</v>
       </c>
       <c r="M16" s="32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N16" s="33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O16" s="32"/>
       <c r="P16" s="32"/>
@@ -3967,10 +3986,10 @@
         <v>12</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N17" s="29" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4006,10 +4025,10 @@
         <v>12</v>
       </c>
       <c r="M18" s="32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N18" s="33" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O18" s="32"/>
       <c r="P18" s="32"/>
@@ -4053,7 +4072,7 @@
         <v>12</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N19" s="11" t="s">
         <v>359</v>
@@ -4094,13 +4113,13 @@
         <v>2</v>
       </c>
       <c r="L20" s="33" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="M20" s="32" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N20" s="33" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="O20" s="32"/>
       <c r="P20" s="32"/>
@@ -4127,7 +4146,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>11</v>
@@ -4146,10 +4165,10 @@
         <v>357</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N21" s="29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4192,10 +4211,10 @@
         <v>12</v>
       </c>
       <c r="M22" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N22" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="O22" s="34"/>
       <c r="P22" s="34"/>
@@ -4241,10 +4260,10 @@
         <v>250</v>
       </c>
       <c r="M23" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N23" s="29" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
@@ -4290,7 +4309,7 @@
         <v>250</v>
       </c>
       <c r="M24" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N24" s="34" t="s">
         <v>359</v>
@@ -4337,10 +4356,10 @@
         <v>250</v>
       </c>
       <c r="M25" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N25" s="29" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="O25" s="29"/>
       <c r="P25" s="29"/>
@@ -4384,7 +4403,7 @@
         <v>12</v>
       </c>
       <c r="M26" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N26" s="34" t="s">
         <v>359</v>
@@ -4431,10 +4450,10 @@
         <v>250</v>
       </c>
       <c r="M27" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N27" s="29" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="O27" s="29"/>
       <c r="P27" s="29"/>
@@ -4480,7 +4499,7 @@
         <v>12</v>
       </c>
       <c r="M28" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N28" s="34" t="s">
         <v>359</v>
@@ -4529,7 +4548,7 @@
         <v>250</v>
       </c>
       <c r="M29" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N29" s="29" t="s">
         <v>359</v>
@@ -4578,7 +4597,7 @@
         <v>250</v>
       </c>
       <c r="M30" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N30" s="34" t="s">
         <v>359</v>
@@ -4625,10 +4644,10 @@
         <v>250</v>
       </c>
       <c r="M31" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N31" s="29" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="O31" s="29"/>
       <c r="P31" s="29"/>
@@ -4655,7 +4674,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="53" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H32" s="34" t="s">
         <v>11</v>
@@ -4674,10 +4693,10 @@
         <v>250</v>
       </c>
       <c r="M32" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N32" s="53" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="O32" s="34"/>
       <c r="P32" s="34"/>
@@ -4704,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H33" s="29" t="s">
         <v>11</v>
@@ -4723,10 +4742,10 @@
         <v>250</v>
       </c>
       <c r="M33" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N33" s="29" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="O33" s="29"/>
       <c r="P33" s="29"/>
@@ -4753,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="34" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H34" s="34" t="s">
         <v>11</v>
@@ -4772,10 +4791,10 @@
         <v>12</v>
       </c>
       <c r="M34" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N34" s="53" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="O34" s="34"/>
       <c r="P34" s="34"/>
@@ -4821,10 +4840,10 @@
         <v>250</v>
       </c>
       <c r="M35" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N35" s="29" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="O35" s="29"/>
       <c r="P35" s="29"/>
@@ -4868,10 +4887,10 @@
         <v>250</v>
       </c>
       <c r="M36" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N36" s="53" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O36" s="34"/>
       <c r="P36" s="34"/>
@@ -4915,10 +4934,10 @@
         <v>250</v>
       </c>
       <c r="M37" s="29" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N37" s="29" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="O37" s="29"/>
       <c r="P37" s="29"/>
@@ -4962,10 +4981,10 @@
         <v>250</v>
       </c>
       <c r="M38" s="37" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N38" s="37" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="O38" s="37"/>
       <c r="P38" s="37"/>
@@ -5011,7 +5030,7 @@
         <v>12</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N39" s="29" t="s">
         <v>359</v>
@@ -5055,10 +5074,10 @@
         <v>250</v>
       </c>
       <c r="M40" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N40" s="39" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O40" s="39"/>
       <c r="P40" s="39"/>
@@ -5104,10 +5123,10 @@
         <v>250</v>
       </c>
       <c r="M41" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N41" s="38" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="O41" s="38"/>
       <c r="P41" s="38"/>
@@ -5153,10 +5172,10 @@
         <v>250</v>
       </c>
       <c r="M42" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N42" s="39" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="O42" s="39"/>
       <c r="P42" s="39"/>
@@ -5199,13 +5218,13 @@
         <v>2</v>
       </c>
       <c r="L43" s="38" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="M43" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N43" s="38" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="O43" s="38"/>
       <c r="P43" s="38"/>
@@ -5235,7 +5254,7 @@
         <v>242</v>
       </c>
       <c r="H44" s="39" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="I44" s="39" t="s">
         <v>11</v>
@@ -5251,10 +5270,10 @@
         <v>250</v>
       </c>
       <c r="M44" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N44" s="39" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="O44" s="39"/>
       <c r="P44" s="39"/>
@@ -5297,13 +5316,13 @@
         <v>3</v>
       </c>
       <c r="L45" s="38" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="M45" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N45" s="38" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O45" s="38"/>
       <c r="P45" s="38"/>
@@ -5349,10 +5368,10 @@
         <v>250</v>
       </c>
       <c r="M46" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N46" s="39" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="O46" s="39"/>
       <c r="P46" s="39"/>
@@ -5398,10 +5417,10 @@
         <v>250</v>
       </c>
       <c r="M47" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N47" s="38" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="O47" s="38"/>
       <c r="P47" s="38"/>
@@ -5447,10 +5466,10 @@
         <v>250</v>
       </c>
       <c r="M48" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N48" s="39" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="O48" s="39"/>
       <c r="P48" s="39"/>
@@ -5496,10 +5515,10 @@
         <v>250</v>
       </c>
       <c r="M49" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N49" s="38" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="O49" s="38"/>
       <c r="P49" s="38"/>
@@ -5545,10 +5564,10 @@
         <v>250</v>
       </c>
       <c r="M50" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N50" s="39" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="O50" s="39"/>
       <c r="P50" s="39"/>
@@ -5592,10 +5611,10 @@
         <v>250</v>
       </c>
       <c r="M51" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N51" s="38" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="O51" s="38"/>
       <c r="P51" s="38"/>
@@ -5637,10 +5656,10 @@
         <v>250</v>
       </c>
       <c r="M52" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N52" s="39" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="O52" s="39"/>
       <c r="P52" s="39"/>
@@ -5682,10 +5701,10 @@
         <v>250</v>
       </c>
       <c r="M53" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N53" s="38" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="O53" s="38"/>
       <c r="P53" s="38"/>
@@ -5729,10 +5748,10 @@
         <v>250</v>
       </c>
       <c r="M54" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N54" s="39" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="O54" s="39"/>
       <c r="P54" s="39"/>
@@ -5776,10 +5795,10 @@
         <v>250</v>
       </c>
       <c r="M55" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N55" s="38" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="O55" s="38"/>
       <c r="P55" s="38"/>
@@ -5822,13 +5841,13 @@
         <v>8</v>
       </c>
       <c r="L56" s="39" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="M56" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N56" s="39" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="O56" s="39"/>
       <c r="P56" s="39"/>
@@ -5874,10 +5893,10 @@
         <v>250</v>
       </c>
       <c r="M57" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N57" s="38" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="O57" s="38"/>
       <c r="P57" s="38"/>
@@ -5923,10 +5942,10 @@
         <v>250</v>
       </c>
       <c r="M58" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N58" s="39" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="O58" s="39"/>
       <c r="P58" s="39"/>
@@ -5964,10 +5983,10 @@
         <v>12</v>
       </c>
       <c r="M59" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N59" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="60" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6004,10 +6023,10 @@
         <v>250</v>
       </c>
       <c r="M60" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N60" s="41" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="O60" s="41"/>
       <c r="P60" s="41"/>
@@ -6049,10 +6068,10 @@
         <v>250</v>
       </c>
       <c r="M61" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N61" s="38" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="O61" s="38"/>
       <c r="P61" s="38"/>
@@ -6094,10 +6113,10 @@
         <v>250</v>
       </c>
       <c r="M62" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N62" s="41" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="O62" s="41"/>
       <c r="P62" s="41"/>
@@ -6137,10 +6156,10 @@
         <v>250</v>
       </c>
       <c r="M63" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N63" s="38" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="O63" s="38"/>
       <c r="P63" s="38"/>
@@ -6180,10 +6199,10 @@
         <v>250</v>
       </c>
       <c r="M64" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N64" s="41" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="O64" s="41"/>
       <c r="P64" s="41"/>
@@ -6223,10 +6242,10 @@
         <v>250</v>
       </c>
       <c r="M65" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N65" s="38" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="O65" s="38"/>
       <c r="P65" s="38"/>
@@ -6266,10 +6285,10 @@
         <v>250</v>
       </c>
       <c r="M66" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N66" s="41" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="O66" s="41"/>
       <c r="P66" s="41"/>
@@ -6309,10 +6328,10 @@
         <v>250</v>
       </c>
       <c r="M67" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N67" s="38" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="O67" s="38"/>
       <c r="P67" s="38"/>
@@ -6352,10 +6371,10 @@
         <v>250</v>
       </c>
       <c r="M68" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N68" s="41" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="O68" s="41"/>
       <c r="P68" s="41"/>
@@ -6395,10 +6414,10 @@
         <v>250</v>
       </c>
       <c r="M69" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N69" s="38" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="O69" s="38"/>
       <c r="P69" s="38"/>
@@ -6438,10 +6457,10 @@
         <v>250</v>
       </c>
       <c r="M70" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N70" s="41" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="O70" s="41"/>
       <c r="P70" s="41"/>
@@ -6483,10 +6502,10 @@
         <v>250</v>
       </c>
       <c r="M71" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N71" s="38" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="O71" s="38"/>
       <c r="P71" s="38"/>
@@ -6526,10 +6545,10 @@
         <v>250</v>
       </c>
       <c r="M72" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N72" s="41" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="O72" s="41"/>
       <c r="P72" s="41"/>
@@ -6571,10 +6590,10 @@
         <v>250</v>
       </c>
       <c r="M73" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N73" s="38" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="O73" s="38"/>
       <c r="P73" s="38"/>
@@ -6618,10 +6637,10 @@
         <v>250</v>
       </c>
       <c r="M74" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N74" s="41" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="O74" s="41"/>
       <c r="P74" s="41"/>
@@ -6665,10 +6684,10 @@
         <v>250</v>
       </c>
       <c r="M75" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N75" s="38" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="O75" s="38"/>
       <c r="P75" s="38"/>
@@ -6707,13 +6726,13 @@
         <v>13</v>
       </c>
       <c r="L76" s="41" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="M76" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N76" s="41" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="O76" s="41"/>
       <c r="P76" s="41"/>
@@ -6753,10 +6772,10 @@
         <v>250</v>
       </c>
       <c r="M77" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N77" s="38" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="O77" s="38"/>
       <c r="P77" s="38"/>
@@ -6798,10 +6817,10 @@
         <v>250</v>
       </c>
       <c r="M78" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N78" s="41" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="O78" s="41"/>
       <c r="P78" s="41"/>
@@ -6841,10 +6860,10 @@
         <v>250</v>
       </c>
       <c r="M79" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N79" s="38" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="O79" s="38"/>
       <c r="P79" s="38"/>
@@ -6884,10 +6903,10 @@
         <v>250</v>
       </c>
       <c r="M80" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N80" s="41" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="O80" s="41"/>
       <c r="P80" s="41"/>
@@ -6924,13 +6943,13 @@
         <v>28</v>
       </c>
       <c r="L81" s="38" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="M81" s="38" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N81" s="38" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="O81" s="38"/>
       <c r="P81" s="38"/>
@@ -6938,14 +6957,14 @@
     </row>
     <row r="82" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="41" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B82" s="41" t="str">
         <f>A82</f>
         <v>Counter-Blade</v>
       </c>
       <c r="C82" s="41" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D82" s="41" t="s">
         <v>228</v>
@@ -6972,10 +6991,10 @@
         <v>250</v>
       </c>
       <c r="M82" s="41" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N82" s="41" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="O82" s="41"/>
       <c r="P82" s="41"/>
@@ -7227,7 +7246,7 @@
         <v>30</v>
       </c>
       <c r="J1" s="56" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>31</v>
@@ -7239,10 +7258,10 @@
         <v>33</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -7271,7 +7290,7 @@
         <v>317</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J2" s="26" t="s">
         <v>317</v>
@@ -7285,7 +7304,7 @@
       <c r="M2" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="59"/>
+      <c r="N2" s="58"/>
       <c r="O2" s="6" t="str">
         <f t="shared" ref="O2:O30" si="0">A3</f>
         <v>1-2</v>
@@ -7317,10 +7336,10 @@
         <v>317</v>
       </c>
       <c r="I3" s="27" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J3" s="27" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="K3" s="16">
         <v>0</v>
@@ -7366,7 +7385,7 @@
         <v>317</v>
       </c>
       <c r="I4" s="26" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>317</v>
@@ -7409,13 +7428,13 @@
         <v>308</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>317</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="J5" s="16" t="s">
         <v>317</v>
@@ -7467,7 +7486,7 @@
         <v>11</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="K6" s="6">
         <v>1</v>
@@ -7476,7 +7495,7 @@
         <v>4</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="N6" s="6" t="str">
         <f t="shared" si="1"/>
@@ -7510,13 +7529,13 @@
         <v>317</v>
       </c>
       <c r="H7" s="27" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I7" s="27" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J7" s="27" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K7" s="16">
         <v>1</v>
@@ -7559,22 +7578,22 @@
         <v>317</v>
       </c>
       <c r="H8" s="52" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I8" s="52" t="s">
         <v>43</v>
       </c>
       <c r="J8" s="52" t="s">
-        <v>445</v>
-      </c>
-      <c r="K8" s="62">
+        <v>444</v>
+      </c>
+      <c r="K8" s="61">
         <v>1</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="61">
         <v>5</v>
       </c>
       <c r="M8" s="52" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="N8" s="52" t="str">
         <f t="shared" si="1"/>
@@ -7611,10 +7630,10 @@
         <v>317</v>
       </c>
       <c r="I9" s="57" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="J9" s="57" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="K9" s="27">
         <v>2</v>
@@ -7653,22 +7672,22 @@
       <c r="F10" s="52" t="s">
         <v>313</v>
       </c>
-      <c r="G10" s="67" t="s">
-        <v>484</v>
+      <c r="G10" s="66" t="s">
+        <v>483</v>
       </c>
       <c r="H10" s="52" t="s">
         <v>317</v>
       </c>
       <c r="I10" s="52" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J10" s="52" t="s">
         <v>317</v>
       </c>
-      <c r="K10" s="62">
+      <c r="K10" s="61">
         <v>2</v>
       </c>
-      <c r="L10" s="62">
+      <c r="L10" s="61">
         <v>6</v>
       </c>
       <c r="M10" s="52" t="s">
@@ -7709,10 +7728,10 @@
         <v>317</v>
       </c>
       <c r="I11" s="57" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K11" s="27">
         <v>3</v>
@@ -7758,15 +7777,15 @@
         <v>317</v>
       </c>
       <c r="I12" s="52" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J12" s="52" t="s">
-        <v>447</v>
-      </c>
-      <c r="K12" s="62">
+        <v>446</v>
+      </c>
+      <c r="K12" s="61">
         <v>3</v>
       </c>
-      <c r="L12" s="62">
+      <c r="L12" s="61">
         <v>7</v>
       </c>
       <c r="M12" s="52" t="s">
@@ -7807,10 +7826,10 @@
         <v>317</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="J13" s="27" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="K13" s="16">
         <v>3</v>
@@ -7818,7 +7837,7 @@
       <c r="L13" s="51">
         <v>7</v>
       </c>
-      <c r="M13" s="63" t="s">
+      <c r="M13" s="62" t="s">
         <v>12</v>
       </c>
       <c r="N13" s="9" t="str">
@@ -7856,10 +7875,10 @@
         <v>317</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="J14" s="33" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="K14" s="33">
         <v>4</v>
@@ -7867,7 +7886,7 @@
       <c r="L14" s="33">
         <v>7</v>
       </c>
-      <c r="M14" s="64" t="s">
+      <c r="M14" s="63" t="s">
         <v>12</v>
       </c>
       <c r="N14" s="33" t="str">
@@ -7905,10 +7924,10 @@
         <v>317</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K15" s="16">
         <v>4</v>
@@ -7957,7 +7976,7 @@
         <v>11</v>
       </c>
       <c r="J16" s="33" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K16" s="33">
         <v>5</v>
@@ -7965,7 +7984,7 @@
       <c r="L16" s="33">
         <v>8</v>
       </c>
-      <c r="M16" s="64" t="s">
+      <c r="M16" s="63" t="s">
         <v>12</v>
       </c>
       <c r="N16" s="33" t="str">
@@ -8003,10 +8022,10 @@
         <v>317</v>
       </c>
       <c r="I17" s="27" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="J17" s="27" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="K17" s="16">
         <v>5</v>
@@ -8052,10 +8071,10 @@
         <v>317</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J18" s="33" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="K18" s="33">
         <v>5</v>
@@ -8063,7 +8082,7 @@
       <c r="L18" s="33">
         <v>9</v>
       </c>
-      <c r="M18" s="64" t="s">
+      <c r="M18" s="63" t="s">
         <v>12</v>
       </c>
       <c r="N18" s="33" t="str">
@@ -8104,7 +8123,7 @@
         <v>317</v>
       </c>
       <c r="J19" s="27" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="K19" s="16">
         <v>6</v>
@@ -8150,10 +8169,10 @@
         <v>317</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J20" s="39" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="K20" s="39">
         <v>6</v>
@@ -8161,7 +8180,7 @@
       <c r="L20" s="39">
         <v>10</v>
       </c>
-      <c r="M20" s="65" t="s">
+      <c r="M20" s="64" t="s">
         <v>12</v>
       </c>
       <c r="N20" s="39" t="str">
@@ -8199,7 +8218,7 @@
         <v>317</v>
       </c>
       <c r="I21" s="27" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>317</v>
@@ -8210,7 +8229,7 @@
       <c r="L21" s="51">
         <v>10</v>
       </c>
-      <c r="M21" s="63" t="s">
+      <c r="M21" s="62" t="s">
         <v>12</v>
       </c>
       <c r="N21" s="9" t="str">
@@ -8248,10 +8267,10 @@
         <v>317</v>
       </c>
       <c r="I22" s="39" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="J22" s="39" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K22" s="39">
         <v>6</v>
@@ -8259,7 +8278,7 @@
       <c r="L22" s="39">
         <v>11</v>
       </c>
-      <c r="M22" s="65" t="s">
+      <c r="M22" s="64" t="s">
         <v>12</v>
       </c>
       <c r="N22" s="39" t="str">
@@ -8300,7 +8319,7 @@
         <v>317</v>
       </c>
       <c r="J23" s="27" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="K23" s="16">
         <v>7</v>
@@ -8308,7 +8327,7 @@
       <c r="L23" s="51">
         <v>12</v>
       </c>
-      <c r="M23" s="63" t="s">
+      <c r="M23" s="62" t="s">
         <v>12</v>
       </c>
       <c r="N23" s="9" t="str">
@@ -8349,7 +8368,7 @@
         <v>317</v>
       </c>
       <c r="J24" s="39" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K24" s="39">
         <v>8</v>
@@ -8357,7 +8376,7 @@
       <c r="L24" s="39">
         <v>12</v>
       </c>
-      <c r="M24" s="65" t="s">
+      <c r="M24" s="64" t="s">
         <v>12</v>
       </c>
       <c r="N24" s="39" t="str">
@@ -8406,7 +8425,7 @@
       <c r="L25" s="51">
         <v>12</v>
       </c>
-      <c r="M25" s="63" t="s">
+      <c r="M25" s="62" t="s">
         <v>12</v>
       </c>
       <c r="N25" s="9" t="str">
@@ -8447,7 +8466,7 @@
         <v>317</v>
       </c>
       <c r="J26" s="41" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="K26" s="41">
         <v>9</v>
@@ -8455,7 +8474,7 @@
       <c r="L26" s="41">
         <v>13</v>
       </c>
-      <c r="M26" s="66" t="s">
+      <c r="M26" s="65" t="s">
         <v>12</v>
       </c>
       <c r="N26" s="41" t="str">
@@ -8493,7 +8512,7 @@
         <v>317</v>
       </c>
       <c r="I27" s="27" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>317</v>
@@ -8535,8 +8554,8 @@
       <c r="F28" s="41" t="s">
         <v>348</v>
       </c>
-      <c r="G28" s="68" t="s">
-        <v>485</v>
+      <c r="G28" s="67" t="s">
+        <v>484</v>
       </c>
       <c r="H28" s="41" t="s">
         <v>317</v>
@@ -8545,7 +8564,7 @@
         <v>11</v>
       </c>
       <c r="J28" s="41" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K28" s="41">
         <v>10</v>
@@ -8553,7 +8572,7 @@
       <c r="L28" s="41">
         <v>14</v>
       </c>
-      <c r="M28" s="66" t="s">
+      <c r="M28" s="65" t="s">
         <v>12</v>
       </c>
       <c r="N28" s="41" t="str">
@@ -8585,7 +8604,7 @@
         <v>349</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="H29" s="16" t="s">
         <v>317</v>
@@ -8594,7 +8613,7 @@
         <v>11</v>
       </c>
       <c r="J29" s="27" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K29" s="16">
         <v>11</v>
@@ -8633,8 +8652,8 @@
       <c r="F30" s="41" t="s">
         <v>350</v>
       </c>
-      <c r="G30" s="68" t="s">
-        <v>485</v>
+      <c r="G30" s="67" t="s">
+        <v>484</v>
       </c>
       <c r="H30" s="41" t="s">
         <v>317</v>
@@ -8643,7 +8662,7 @@
         <v>11</v>
       </c>
       <c r="J30" s="41" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K30" s="41">
         <v>12</v>
@@ -8651,7 +8670,7 @@
       <c r="L30" s="41">
         <v>14</v>
       </c>
-      <c r="M30" s="66" t="s">
+      <c r="M30" s="65" t="s">
         <v>12</v>
       </c>
       <c r="N30" s="41" t="str">
@@ -8683,7 +8702,7 @@
         <v>351</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>317</v>
@@ -8692,7 +8711,7 @@
         <v>11</v>
       </c>
       <c r="J31" s="27" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K31" s="16">
         <v>12</v>
@@ -8707,7 +8726,7 @@
         <f t="shared" si="1"/>
         <v>5-5</v>
       </c>
-      <c r="O31" s="60"/>
+      <c r="O31" s="59"/>
     </row>
     <row r="32" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="25"/>

</xml_diff>